<commit_message>
add week 4 and 5
</commit_message>
<xml_diff>
--- a/Woche03/2026-10-14/[PRACTICE] SUMMEWENN.xlsx
+++ b/Woche03/2026-10-14/[PRACTICE] SUMMEWENN.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://dsinstitute-my.sharepoint.com/personal/yannik_rohrschneider_dsinstitute_de/Documents/Dokumente/Lehre/Excel/W3/01/Nachmittag/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\DSI\Python\Woche03\2026-10-14\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="73" documentId="13_ncr:1_{92C5B1CB-AEC4-4756-A8DF-725FDF5A12D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{10EF094A-5DE0-4C18-9E75-D35807341A76}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{48773371-51AE-470D-9E12-D09D5C7948A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{A452F4AE-B2D0-430D-ACDA-315AA4B42298}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{A452F4AE-B2D0-430D-ACDA-315AA4B42298}"/>
   </bookViews>
   <sheets>
     <sheet name="Aufgaben" sheetId="2" r:id="rId1"/>
@@ -51,7 +51,8 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Segoe UI"/>
-            <charset val="1"/>
+            <family val="2"/>
+            <charset val="204"/>
           </rPr>
           <t>Das * enthält beliebig viele Buchstaben. Mit "A*" finden wir also alle Wörter, die mit "A" beginnen.</t>
         </r>
@@ -761,7 +762,8 @@
       <sz val="9"/>
       <color indexed="81"/>
       <name val="Segoe UI"/>
-      <charset val="1"/>
+      <family val="2"/>
+      <charset val="204"/>
     </font>
   </fonts>
   <fills count="5">
@@ -1033,9 +1035,9 @@
     </xf>
   </cellXfs>
   <cellStyles count="3">
-    <cellStyle name="Prozent" xfId="1" builtinId="5"/>
-    <cellStyle name="Standard" xfId="0" builtinId="0"/>
-    <cellStyle name="Überschrift 2" xfId="2" builtinId="17"/>
+    <cellStyle name="Відсотковий" xfId="1" builtinId="5"/>
+    <cellStyle name="Заголовок 2" xfId="2" builtinId="17"/>
+    <cellStyle name="Звичайний" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="19">
     <dxf>
@@ -1812,16 +1814,16 @@
     <tableColumn id="5" xr3:uid="{429633E8-C9EC-4837-B13A-0F3574E29E81}" name="Brand" dataDxfId="3"/>
     <tableColumn id="6" xr3:uid="{FD92F6B7-94AB-4799-8CD1-1C1E89862EA0}" name="Cost Price" dataDxfId="2"/>
     <tableColumn id="7" xr3:uid="{CAA6CD8E-9A96-48A7-B8D6-4A8DD1B7DE6B}" name="Selling Price" dataDxfId="1"/>
-    <tableColumn id="8" xr3:uid="{4612EDD6-A50B-4293-98F5-A4F62F7C25F5}" name="Profit %" dataDxfId="0" dataCellStyle="Prozent"/>
+    <tableColumn id="8" xr3:uid="{4612EDD6-A50B-4293-98F5-A4F62F7C25F5}" name="Profit %" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Тема Office">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Офіс">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1859,7 +1861,7 @@
         <a:srgbClr val="96607D"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Офіс">
       <a:majorFont>
         <a:latin typeface="Aptos Display" panose="02110004020202020204"/>
         <a:ea typeface=""/>
@@ -1965,7 +1967,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Офіс">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -2136,32 +2138,32 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C9B81E2F-828D-4CD0-95A3-41BD54594486}">
   <dimension ref="A1:L93"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="3.7109375" style="1" customWidth="1"/>
+    <col min="1" max="1" width="3.7265625" style="1" customWidth="1"/>
     <col min="2" max="2" width="5" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.7109375" style="1" customWidth="1"/>
-    <col min="5" max="5" width="21.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9.85546875" style="1" customWidth="1"/>
-    <col min="7" max="7" width="14.42578125" style="1" customWidth="1"/>
-    <col min="8" max="8" width="16.7109375" style="1" customWidth="1"/>
-    <col min="9" max="9" width="11.5703125" style="1" customWidth="1"/>
-    <col min="10" max="10" width="5.28515625" style="1" customWidth="1"/>
-    <col min="11" max="11" width="32.28515625" style="1" customWidth="1"/>
-    <col min="12" max="12" width="32.7109375" style="1" customWidth="1"/>
-    <col min="13" max="15" width="9.140625" style="1"/>
-    <col min="16" max="16" width="13.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="12.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="18" max="16384" width="9.140625" style="1"/>
+    <col min="3" max="3" width="10.54296875" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.7265625" style="1" customWidth="1"/>
+    <col min="5" max="5" width="21.81640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.81640625" style="1" customWidth="1"/>
+    <col min="7" max="7" width="14.453125" style="1" customWidth="1"/>
+    <col min="8" max="8" width="16.7265625" style="1" customWidth="1"/>
+    <col min="9" max="9" width="11.54296875" style="1" customWidth="1"/>
+    <col min="10" max="10" width="5.26953125" style="1" customWidth="1"/>
+    <col min="11" max="11" width="32.26953125" style="1" customWidth="1"/>
+    <col min="12" max="12" width="32.7265625" style="1" customWidth="1"/>
+    <col min="13" max="15" width="9.1796875" style="1"/>
+    <col min="16" max="16" width="13.7265625" style="1" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="12.453125" style="1" bestFit="1" customWidth="1"/>
+    <col min="18" max="16384" width="9.1796875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>208</v>
       </c>
     </row>
-    <row r="2" spans="1:12" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:12" ht="20.149999999999999" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B2" s="30" t="s">
         <v>0</v>
       </c>
@@ -2173,8 +2175,8 @@
       <c r="H2" s="30"/>
       <c r="I2" s="30"/>
     </row>
-    <row r="3" spans="1:12" ht="20.100000000000001" customHeight="1" thickTop="1" x14ac:dyDescent="0.25"/>
-    <row r="5" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:12" ht="20.149999999999999" customHeight="1" thickTop="1" x14ac:dyDescent="0.35"/>
+    <row r="5" spans="1:12" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B5" s="27" t="s">
         <v>1</v>
       </c>
@@ -2203,7 +2205,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="6" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:12" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B6" s="18" t="s">
         <v>10</v>
       </c>
@@ -2232,9 +2234,12 @@
       <c r="K6" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="L6" s="6"/>
-    </row>
-    <row r="7" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L6" s="6">
+        <f>SUMIF(G6:G93, "&gt;1000")</f>
+        <v>79327.760000000009</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B7" s="19" t="s">
         <v>15</v>
       </c>
@@ -2261,7 +2266,7 @@
       </c>
       <c r="J7" s="5"/>
     </row>
-    <row r="8" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:12" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B8" s="18" t="s">
         <v>19</v>
       </c>
@@ -2292,7 +2297,7 @@
       </c>
       <c r="L8" s="7"/>
     </row>
-    <row r="9" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:12" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B9" s="19" t="s">
         <v>21</v>
       </c>
@@ -2321,9 +2326,12 @@
       <c r="K9" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="L9" s="6"/>
-    </row>
-    <row r="10" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L9" s="6">
+        <f>SUMIF(D6:D93, "Ben", H6:H93)</f>
+        <v>56779.25</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B10" s="18" t="s">
         <v>24</v>
       </c>
@@ -2352,9 +2360,12 @@
       <c r="K10" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="L10" s="6"/>
-    </row>
-    <row r="11" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L10" s="6">
+        <f>SUMIF(D6:D93, "Jacob", H6:H93)</f>
+        <v>56646.5</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B11" s="19" t="s">
         <v>27</v>
       </c>
@@ -2381,7 +2392,7 @@
       </c>
       <c r="J11" s="5"/>
     </row>
-    <row r="12" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:12" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B12" s="18" t="s">
         <v>30</v>
       </c>
@@ -2412,7 +2423,7 @@
       </c>
       <c r="L12" s="7"/>
     </row>
-    <row r="13" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:12" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B13" s="19" t="s">
         <v>33</v>
       </c>
@@ -2441,9 +2452,12 @@
       <c r="K13" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="L13" s="4"/>
-    </row>
-    <row r="14" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L13" s="4">
+        <f>SUMIF(F6:F93, "A*", H6:H93)</f>
+        <v>28483.75</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B14" s="18" t="s">
         <v>36</v>
       </c>
@@ -2470,7 +2484,7 @@
       </c>
       <c r="J14" s="5"/>
     </row>
-    <row r="15" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:12" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B15" s="19" t="s">
         <v>39</v>
       </c>
@@ -2500,7 +2514,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="16" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:12" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B16" s="18" t="s">
         <v>42</v>
       </c>
@@ -2529,9 +2543,12 @@
       <c r="K16" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="L16" s="4"/>
-    </row>
-    <row r="17" spans="2:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L16" s="4">
+        <f>SUMIF(F6:F93, "Sony", H6:H93) + SUMIF(F6:F93, "Acer", H6:H93)</f>
+        <v>31082.5</v>
+      </c>
+    </row>
+    <row r="17" spans="2:12" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B17" s="19" t="s">
         <v>45</v>
       </c>
@@ -2558,7 +2575,7 @@
       </c>
       <c r="J17" s="5"/>
     </row>
-    <row r="18" spans="2:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:12" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B18" s="18" t="s">
         <v>47</v>
       </c>
@@ -2588,7 +2605,7 @@
         <v>207</v>
       </c>
     </row>
-    <row r="19" spans="2:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:12" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B19" s="19" t="s">
         <v>49</v>
       </c>
@@ -2617,9 +2634,12 @@
       <c r="K19" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="L19" s="4"/>
-    </row>
-    <row r="20" spans="2:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L19" s="4">
+        <f>SUMIFS(H6:H93, C6:C93, "&gt;=01.07.2022", C6:C93, "&lt;=31.07.2022") - SUMIFS(G6:G93, C6:C93, "&gt;=01.07.2022", C6:C93, "&lt;=31.07.2022")</f>
+        <v>5165.0799999999945</v>
+      </c>
+    </row>
+    <row r="20" spans="2:12" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B20" s="18" t="s">
         <v>53</v>
       </c>
@@ -2646,7 +2666,7 @@
       </c>
       <c r="J20" s="5"/>
     </row>
-    <row r="21" spans="2:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:12" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B21" s="19" t="s">
         <v>56</v>
       </c>
@@ -2673,7 +2693,7 @@
       </c>
       <c r="J21" s="5"/>
     </row>
-    <row r="22" spans="2:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:12" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B22" s="18" t="s">
         <v>58</v>
       </c>
@@ -2700,7 +2720,7 @@
       </c>
       <c r="J22" s="5"/>
     </row>
-    <row r="23" spans="2:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:12" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B23" s="19" t="s">
         <v>61</v>
       </c>
@@ -2727,7 +2747,7 @@
       </c>
       <c r="J23" s="5"/>
     </row>
-    <row r="24" spans="2:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:12" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B24" s="18" t="s">
         <v>63</v>
       </c>
@@ -2754,7 +2774,7 @@
       </c>
       <c r="J24" s="5"/>
     </row>
-    <row r="25" spans="2:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:12" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B25" s="19" t="s">
         <v>65</v>
       </c>
@@ -2781,7 +2801,7 @@
       </c>
       <c r="J25" s="5"/>
     </row>
-    <row r="26" spans="2:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:12" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B26" s="18" t="s">
         <v>67</v>
       </c>
@@ -2808,7 +2828,7 @@
       </c>
       <c r="J26" s="5"/>
     </row>
-    <row r="27" spans="2:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:12" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B27" s="19" t="s">
         <v>69</v>
       </c>
@@ -2835,7 +2855,7 @@
       </c>
       <c r="J27" s="5"/>
     </row>
-    <row r="28" spans="2:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:12" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B28" s="18" t="s">
         <v>71</v>
       </c>
@@ -2862,7 +2882,7 @@
       </c>
       <c r="J28" s="5"/>
     </row>
-    <row r="29" spans="2:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:12" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B29" s="19" t="s">
         <v>73</v>
       </c>
@@ -2889,7 +2909,7 @@
       </c>
       <c r="J29" s="5"/>
     </row>
-    <row r="30" spans="2:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:12" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B30" s="18" t="s">
         <v>75</v>
       </c>
@@ -2916,7 +2936,7 @@
       </c>
       <c r="J30" s="5"/>
     </row>
-    <row r="31" spans="2:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="2:12" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B31" s="19" t="s">
         <v>77</v>
       </c>
@@ -2943,7 +2963,7 @@
       </c>
       <c r="J31" s="5"/>
     </row>
-    <row r="32" spans="2:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:12" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B32" s="18" t="s">
         <v>79</v>
       </c>
@@ -2970,7 +2990,7 @@
       </c>
       <c r="J32" s="5"/>
     </row>
-    <row r="33" spans="2:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="2:10" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B33" s="19" t="s">
         <v>81</v>
       </c>
@@ -2997,7 +3017,7 @@
       </c>
       <c r="J33" s="5"/>
     </row>
-    <row r="34" spans="2:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="2:10" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B34" s="18" t="s">
         <v>83</v>
       </c>
@@ -3024,7 +3044,7 @@
       </c>
       <c r="J34" s="5"/>
     </row>
-    <row r="35" spans="2:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:10" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B35" s="19" t="s">
         <v>85</v>
       </c>
@@ -3051,7 +3071,7 @@
       </c>
       <c r="J35" s="5"/>
     </row>
-    <row r="36" spans="2:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="2:10" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B36" s="18" t="s">
         <v>87</v>
       </c>
@@ -3078,7 +3098,7 @@
       </c>
       <c r="J36" s="5"/>
     </row>
-    <row r="37" spans="2:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="2:10" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B37" s="19" t="s">
         <v>89</v>
       </c>
@@ -3105,7 +3125,7 @@
       </c>
       <c r="J37" s="5"/>
     </row>
-    <row r="38" spans="2:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="2:10" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B38" s="18" t="s">
         <v>91</v>
       </c>
@@ -3132,7 +3152,7 @@
       </c>
       <c r="J38" s="5"/>
     </row>
-    <row r="39" spans="2:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="2:10" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B39" s="19" t="s">
         <v>93</v>
       </c>
@@ -3159,7 +3179,7 @@
       </c>
       <c r="J39" s="5"/>
     </row>
-    <row r="40" spans="2:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="2:10" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B40" s="18" t="s">
         <v>95</v>
       </c>
@@ -3186,7 +3206,7 @@
       </c>
       <c r="J40" s="5"/>
     </row>
-    <row r="41" spans="2:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="2:10" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B41" s="19" t="s">
         <v>97</v>
       </c>
@@ -3213,7 +3233,7 @@
       </c>
       <c r="J41" s="5"/>
     </row>
-    <row r="42" spans="2:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="2:10" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B42" s="18" t="s">
         <v>99</v>
       </c>
@@ -3240,7 +3260,7 @@
       </c>
       <c r="J42" s="5"/>
     </row>
-    <row r="43" spans="2:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="2:10" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B43" s="19" t="s">
         <v>101</v>
       </c>
@@ -3267,7 +3287,7 @@
       </c>
       <c r="J43" s="5"/>
     </row>
-    <row r="44" spans="2:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="2:10" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B44" s="18" t="s">
         <v>103</v>
       </c>
@@ -3294,7 +3314,7 @@
       </c>
       <c r="J44" s="5"/>
     </row>
-    <row r="45" spans="2:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="2:10" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B45" s="19" t="s">
         <v>105</v>
       </c>
@@ -3321,7 +3341,7 @@
       </c>
       <c r="J45" s="5"/>
     </row>
-    <row r="46" spans="2:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="2:10" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B46" s="18" t="s">
         <v>107</v>
       </c>
@@ -3348,7 +3368,7 @@
       </c>
       <c r="J46" s="5"/>
     </row>
-    <row r="47" spans="2:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="2:10" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B47" s="19" t="s">
         <v>109</v>
       </c>
@@ -3375,7 +3395,7 @@
       </c>
       <c r="J47" s="5"/>
     </row>
-    <row r="48" spans="2:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="2:10" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B48" s="18" t="s">
         <v>111</v>
       </c>
@@ -3402,7 +3422,7 @@
       </c>
       <c r="J48" s="5"/>
     </row>
-    <row r="49" spans="2:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="2:10" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B49" s="19" t="s">
         <v>113</v>
       </c>
@@ -3429,7 +3449,7 @@
       </c>
       <c r="J49" s="5"/>
     </row>
-    <row r="50" spans="2:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="2:10" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B50" s="18" t="s">
         <v>115</v>
       </c>
@@ -3456,7 +3476,7 @@
       </c>
       <c r="J50" s="5"/>
     </row>
-    <row r="51" spans="2:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="51" spans="2:10" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B51" s="19" t="s">
         <v>117</v>
       </c>
@@ -3483,7 +3503,7 @@
       </c>
       <c r="J51" s="5"/>
     </row>
-    <row r="52" spans="2:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="52" spans="2:10" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B52" s="18" t="s">
         <v>119</v>
       </c>
@@ -3510,7 +3530,7 @@
       </c>
       <c r="J52" s="5"/>
     </row>
-    <row r="53" spans="2:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="53" spans="2:10" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B53" s="19" t="s">
         <v>121</v>
       </c>
@@ -3537,7 +3557,7 @@
       </c>
       <c r="J53" s="5"/>
     </row>
-    <row r="54" spans="2:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="54" spans="2:10" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B54" s="18" t="s">
         <v>123</v>
       </c>
@@ -3564,7 +3584,7 @@
       </c>
       <c r="J54" s="5"/>
     </row>
-    <row r="55" spans="2:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="55" spans="2:10" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B55" s="19" t="s">
         <v>125</v>
       </c>
@@ -3591,7 +3611,7 @@
       </c>
       <c r="J55" s="5"/>
     </row>
-    <row r="56" spans="2:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="56" spans="2:10" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B56" s="18" t="s">
         <v>128</v>
       </c>
@@ -3618,7 +3638,7 @@
       </c>
       <c r="J56" s="5"/>
     </row>
-    <row r="57" spans="2:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="57" spans="2:10" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B57" s="19" t="s">
         <v>130</v>
       </c>
@@ -3645,7 +3665,7 @@
       </c>
       <c r="J57" s="5"/>
     </row>
-    <row r="58" spans="2:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="58" spans="2:10" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B58" s="18" t="s">
         <v>132</v>
       </c>
@@ -3672,7 +3692,7 @@
       </c>
       <c r="J58" s="5"/>
     </row>
-    <row r="59" spans="2:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="59" spans="2:10" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B59" s="19" t="s">
         <v>134</v>
       </c>
@@ -3699,7 +3719,7 @@
       </c>
       <c r="J59" s="5"/>
     </row>
-    <row r="60" spans="2:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="60" spans="2:10" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B60" s="18" t="s">
         <v>136</v>
       </c>
@@ -3726,7 +3746,7 @@
       </c>
       <c r="J60" s="5"/>
     </row>
-    <row r="61" spans="2:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="61" spans="2:10" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B61" s="19" t="s">
         <v>138</v>
       </c>
@@ -3753,7 +3773,7 @@
       </c>
       <c r="J61" s="5"/>
     </row>
-    <row r="62" spans="2:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="62" spans="2:10" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B62" s="18" t="s">
         <v>140</v>
       </c>
@@ -3780,7 +3800,7 @@
       </c>
       <c r="J62" s="5"/>
     </row>
-    <row r="63" spans="2:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="63" spans="2:10" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B63" s="19" t="s">
         <v>142</v>
       </c>
@@ -3807,7 +3827,7 @@
       </c>
       <c r="J63" s="5"/>
     </row>
-    <row r="64" spans="2:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="64" spans="2:10" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B64" s="18" t="s">
         <v>144</v>
       </c>
@@ -3834,7 +3854,7 @@
       </c>
       <c r="J64" s="5"/>
     </row>
-    <row r="65" spans="2:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="65" spans="2:10" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B65" s="19" t="s">
         <v>146</v>
       </c>
@@ -3861,7 +3881,7 @@
       </c>
       <c r="J65" s="5"/>
     </row>
-    <row r="66" spans="2:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="66" spans="2:10" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B66" s="18" t="s">
         <v>148</v>
       </c>
@@ -3888,7 +3908,7 @@
       </c>
       <c r="J66" s="5"/>
     </row>
-    <row r="67" spans="2:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="67" spans="2:10" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B67" s="19" t="s">
         <v>150</v>
       </c>
@@ -3915,7 +3935,7 @@
       </c>
       <c r="J67" s="5"/>
     </row>
-    <row r="68" spans="2:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="68" spans="2:10" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B68" s="18" t="s">
         <v>152</v>
       </c>
@@ -3942,7 +3962,7 @@
       </c>
       <c r="J68" s="5"/>
     </row>
-    <row r="69" spans="2:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="69" spans="2:10" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B69" s="19" t="s">
         <v>154</v>
       </c>
@@ -3969,7 +3989,7 @@
       </c>
       <c r="J69" s="5"/>
     </row>
-    <row r="70" spans="2:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="70" spans="2:10" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B70" s="18" t="s">
         <v>156</v>
       </c>
@@ -3996,7 +4016,7 @@
       </c>
       <c r="J70" s="5"/>
     </row>
-    <row r="71" spans="2:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="71" spans="2:10" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B71" s="19" t="s">
         <v>158</v>
       </c>
@@ -4023,7 +4043,7 @@
       </c>
       <c r="J71" s="5"/>
     </row>
-    <row r="72" spans="2:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="72" spans="2:10" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B72" s="18" t="s">
         <v>160</v>
       </c>
@@ -4050,7 +4070,7 @@
       </c>
       <c r="J72" s="5"/>
     </row>
-    <row r="73" spans="2:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="73" spans="2:10" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B73" s="19" t="s">
         <v>162</v>
       </c>
@@ -4077,7 +4097,7 @@
       </c>
       <c r="J73" s="5"/>
     </row>
-    <row r="74" spans="2:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="74" spans="2:10" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B74" s="18" t="s">
         <v>164</v>
       </c>
@@ -4104,7 +4124,7 @@
       </c>
       <c r="J74" s="5"/>
     </row>
-    <row r="75" spans="2:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="75" spans="2:10" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B75" s="19" t="s">
         <v>166</v>
       </c>
@@ -4131,7 +4151,7 @@
       </c>
       <c r="J75" s="5"/>
     </row>
-    <row r="76" spans="2:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="76" spans="2:10" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B76" s="18" t="s">
         <v>168</v>
       </c>
@@ -4158,7 +4178,7 @@
       </c>
       <c r="J76" s="5"/>
     </row>
-    <row r="77" spans="2:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="77" spans="2:10" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B77" s="19" t="s">
         <v>170</v>
       </c>
@@ -4185,7 +4205,7 @@
       </c>
       <c r="J77" s="5"/>
     </row>
-    <row r="78" spans="2:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="78" spans="2:10" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B78" s="18" t="s">
         <v>172</v>
       </c>
@@ -4212,7 +4232,7 @@
       </c>
       <c r="J78" s="5"/>
     </row>
-    <row r="79" spans="2:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="79" spans="2:10" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B79" s="19" t="s">
         <v>174</v>
       </c>
@@ -4239,7 +4259,7 @@
       </c>
       <c r="J79" s="5"/>
     </row>
-    <row r="80" spans="2:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="80" spans="2:10" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B80" s="18" t="s">
         <v>176</v>
       </c>
@@ -4266,7 +4286,7 @@
       </c>
       <c r="J80" s="5"/>
     </row>
-    <row r="81" spans="2:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="81" spans="2:10" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B81" s="19" t="s">
         <v>178</v>
       </c>
@@ -4293,7 +4313,7 @@
       </c>
       <c r="J81" s="5"/>
     </row>
-    <row r="82" spans="2:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="82" spans="2:10" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B82" s="18" t="s">
         <v>180</v>
       </c>
@@ -4320,7 +4340,7 @@
       </c>
       <c r="J82" s="5"/>
     </row>
-    <row r="83" spans="2:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="83" spans="2:10" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B83" s="19" t="s">
         <v>182</v>
       </c>
@@ -4347,7 +4367,7 @@
       </c>
       <c r="J83" s="5"/>
     </row>
-    <row r="84" spans="2:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="84" spans="2:10" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B84" s="18" t="s">
         <v>184</v>
       </c>
@@ -4374,7 +4394,7 @@
       </c>
       <c r="J84" s="5"/>
     </row>
-    <row r="85" spans="2:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="85" spans="2:10" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B85" s="19" t="s">
         <v>186</v>
       </c>
@@ -4401,7 +4421,7 @@
       </c>
       <c r="J85" s="5"/>
     </row>
-    <row r="86" spans="2:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="86" spans="2:10" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B86" s="18" t="s">
         <v>188</v>
       </c>
@@ -4428,7 +4448,7 @@
       </c>
       <c r="J86" s="5"/>
     </row>
-    <row r="87" spans="2:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="87" spans="2:10" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B87" s="19" t="s">
         <v>190</v>
       </c>
@@ -4455,7 +4475,7 @@
       </c>
       <c r="J87" s="5"/>
     </row>
-    <row r="88" spans="2:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="88" spans="2:10" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B88" s="18" t="s">
         <v>192</v>
       </c>
@@ -4482,7 +4502,7 @@
       </c>
       <c r="J88" s="5"/>
     </row>
-    <row r="89" spans="2:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="89" spans="2:10" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B89" s="19" t="s">
         <v>194</v>
       </c>
@@ -4509,7 +4529,7 @@
       </c>
       <c r="J89" s="5"/>
     </row>
-    <row r="90" spans="2:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="90" spans="2:10" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B90" s="18" t="s">
         <v>196</v>
       </c>
@@ -4536,7 +4556,7 @@
       </c>
       <c r="J90" s="5"/>
     </row>
-    <row r="91" spans="2:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="91" spans="2:10" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B91" s="19" t="s">
         <v>198</v>
       </c>
@@ -4563,7 +4583,7 @@
       </c>
       <c r="J91" s="5"/>
     </row>
-    <row r="92" spans="2:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="92" spans="2:10" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B92" s="18" t="s">
         <v>200</v>
       </c>
@@ -4590,7 +4610,7 @@
       </c>
       <c r="J92" s="5"/>
     </row>
-    <row r="93" spans="2:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="93" spans="2:10" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B93" s="22" t="s">
         <v>202</v>
       </c>

</xml_diff>